<commit_message>
Limpieza de archivos obsoletos y fix de errores de lógica y sintaxis
</commit_message>
<xml_diff>
--- a/Presencialidad 2C 2026.xlsx
+++ b/Presencialidad 2C 2026.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27947" windowHeight="12240" tabRatio="500"/>
+    <workbookView windowWidth="27947" windowHeight="11640" tabRatio="500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -241,7 +241,7 @@
     <t>Análisis de Sistemas</t>
   </si>
   <si>
-    <t>Perez</t>
+    <t>Mendez</t>
   </si>
   <si>
     <t>Diseño e Implementación de Pruebas de Software</t>
@@ -2341,8 +2341,6 @@
       <c r="F30" t="s">
         <v>93</v>
       </c>
-      <c r="G30"/>
-      <c r="H30"/>
       <c r="I30" t="s">
         <v>92</v>
       </c>

</xml_diff>